<commit_message>
Add early-cycle setup E (deep fibo + low weekly RSI + fresh MCDX/breakout)
Screens for bottoming stocks on a relaxed-liquidity universe: retraced
past 50 percent of the 240-day range, weekly RSI under 55, MCDX red band
just appearing, first breakout signal within 10 bars and price not yet
extended, ranked by an early-cycle score with its own report sheet.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019R5LS1R4wzyzRwWCixKCHp
</commit_message>
<xml_diff>
--- a/stock-screener/output/watchlist_20260730.xlsx
+++ b/stock-screener/output/watchlist_20260730.xlsx
@@ -14,7 +14,8 @@
     <sheet name="B-Breakout" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="C-Pullback" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="D-MCDX เจ้าเก็บของ" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ย้ายโซน RSI" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="E-ต้นรอบ" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ย้ายโซน RSI" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +53,14 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007C3A00"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +75,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007C3A00"/>
       </patternFill>
     </fill>
     <fill>
@@ -107,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -125,10 +137,14 @@
     <xf numFmtId="4" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -494,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -600,102 +616,114 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t>E-ต้นรอบ (5 ตัว)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ย่อลึกเกิน 50% ของรอบ 240 วัน (หรือ 61.8% ของ 120 วัน) + RSI สัปดาห์ &lt; 55 + MCDX แถบแดงเริ่มโผล่ + เพิ่งมีสัญญาณเบรกแรกภายใน 10 แท่ง (ทะลุ high 10-25 วัน / CDC / MACD / EMA26) + ยังไม่ยืดเกิน 8% | ใช้ universe ผ่อนสภาพคล่อง (≥5 ลบ./วัน, Mcap ≥2 พันลบ.) เพราะก้นรอบวอลุ่มมักเบา — ไม้เล็ก รอวอลุ่มยืนยันก่อนเพิ่ม</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
           <t>คะแนนรวม (composite)</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>SCORE จากไฟล์ 25% + RS rank 20/60 วัน 30% + ADX 10 + RSI สัปดาห์ 5 + MACD เร่งขึ้น 5 + วอลุ่มเข้า 10 + แรงซื้อรายใหญ่ MCDX 10 − โทษ divergence/ยืดตัว</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>โซน RSI (RSIzone)</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>zone1 = RSI วัน&lt;50 และสัปดาห์&lt;50 (อ่อนทั้งคู่) | zone2 = วัน&gt;50 สัปดาห์&lt;50 (เด้งระยะสั้น) | zone3 = &gt;50 ทั้งคู่ (แข็งสุด) | zone4 = วัน&lt;50 สัปดาห์&gt;50 (ย่อในขาขึ้นใหญ่ — โซนตั้งรับ)</t>
-        </is>
-      </c>
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>ชีท "ย้ายโซน RSI"</t>
+          <t>โซน RSI (RSIzone)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>หุ้นที่โซนเพิ่งเปลี่ยนในแท่งล่าสุด — แถวเขียว = ย้ายขึ้น (ฟื้นตัว เช่น zone1→2, zone2→3, zone4→3) | แถวแดง = ย้ายลง (อ่อนแรง เช่น zone3→1, zone3→4) ใช้เตือนทั้งหาจังหวะเข้าและระวังตัวที่ถืออยู่</t>
+          <t>zone1 = RSI วัน&lt;50 และสัปดาห์&lt;50 (อ่อนทั้งคู่) | zone2 = วัน&gt;50 สัปดาห์&lt;50 (เด้งระยะสั้น) | zone3 = &gt;50 ทั้งคู่ (แข็งสุด) | zone4 = วัน&lt;50 สัปดาห์&gt;50 (ย่อในขาขึ้นใหญ่ — โซนตั้งรับ)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>MCDX ในตาราง</t>
+          <t>ชีท "ย้ายโซน RSI"</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>คอลัมน์ "MCDX แดง" = แรงรายใหญ่ล่าสุด (ยิ่งสูงยิ่งเข้าเยอะ, ≥10 = ชัดเจน) | "ΔMCDX 5 แท่ง" = เปลี่ยนแปลง 5 วัน บวก = กำลังเก็บเพิ่ม ลบมาก (≤ -8) = แผ่วลง มีธงเตือนให้</t>
+          <t>หุ้นที่โซนเพิ่งเปลี่ยนในแท่งล่าสุด — แถวเขียว = ย้ายขึ้น (ฟื้นตัว เช่น zone1→2, zone2→3, zone4→3) | แถวแดง = ย้ายลง (อ่อนแรง เช่น zone3→1, zone3→4) ใช้เตือนทั้งหาจังหวะเข้าและระวังตัวที่ถืออยู่</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>MCDX ในตาราง</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>คอลัมน์ "MCDX แดง" = แรงรายใหญ่ล่าสุด (ยิ่งสูงยิ่งเข้าเยอะ, ≥10 = ชัดเจน) | "ΔMCDX 5 แท่ง" = เปลี่ยนแปลง 5 วัน บวก = กำลังเก็บเพิ่ม ลบมาก (≤ -8) = แผ่วลง มีธงเตือนให้</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>ชีท "ภาพตลาด &amp; กลุ่ม"</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Breadth ของทั้งตลาด (% เหนือ MA ต่างๆ, A/D, new high/low) + สรุปโหมดตลาด และตารางแรงหมุนรายกลุ่ม | คอลัมน์ "ชนะกลุ่ม 20 วัน %" ในทุกตาราง = ผลตอบแทนหุ้น ลบ มัธยฐานของกลุ่มตัวเอง (บวก = นำกลุ่ม) เป็นข้อมูลประกอบ ไม่ถูกนำไปคิดในคะแนนรวม</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>การใช้งาน</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>จุดตัดขาดทุนอ้างอิง 2×ATR ใต้ราคาปิด หรือใต้แนวรับ EMA26 — เลือกอันที่ตื้นกว่าตามสไตล์ | ขนาดไม้: เสี่ยงต่อไม้ ~1-2% ของพอร์ต ÷ ระยะถึงจุดตัด</t>
-        </is>
-      </c>
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>คำเตือนสำคัญ</t>
+          <t>การใช้งาน</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>หุ้นที่มี "งบออกใน N วัน" มีความเสี่ยงราคากระโดดข้ามคืนช่วงประกาศงบ ควรลดขนาดไม้หรือรอผ่านงบ</t>
+          <t>จุดตัดขาดทุนอ้างอิง 2×ATR ใต้ราคาปิด หรือใต้แนวรับ EMA26 — เลือกอันที่ตื้นกว่าตามสไตล์ | ขนาดไม้: เสี่ยงต่อไม้ ~1-2% ของพอร์ต ÷ ระยะถึงจุดตัด</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>คำเตือนสำคัญ</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>หุ้นที่มี "งบออกใน N วัน" มีความเสี่ยงราคากระโดดข้ามคืนช่วงประกาศงบ ควรลดขนาดไม้หรือรอผ่านงบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>ข้อจำกัด</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>เป็นการคัดกรองทางเทคนิคจากข้อมูลในไฟล์เท่านั้น ไม่ใช่คำแนะนำการลงทุน ผลในอดีตไม่การันตีอนาคต โปรดพิจารณาปัจจัยพื้นฐาน/ข่าวประกอบและรับความเสี่ยงได้ก่อนเทรดจริง</t>
         </is>
@@ -11598,6 +11626,516 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:U7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>E-ต้นรอบ: เข้าสวนเทรนด์ระยะกลาง — อัตราล้มเหลวสูงกว่ากลยุทธ์ตามเทรนด์ ใช้ไม้เล็ก (pilot) ตัดขาดทุนเคร่งครัด แล้วค่อยเพิ่มไม้เมื่อวอลุ่มและ MCDX มายืนยัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>หุ้น</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>ราคาปิด</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>คะแนนต้นรอบ</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>ย่อจาก high 240 วัน %</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>ย่อจาก high 120 วัน %</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>โซน RSI</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>ย้ายโซน</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>RSI วัน</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>RSI สัปดาห์</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr">
+        <is>
+          <t>MCDX แดง</t>
+        </is>
+      </c>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>ΔMCDX 5 แท่ง</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="inlineStr">
+        <is>
+          <t>วอลุ่ม/เฉลี่ย 25 วัน (เท่า)</t>
+        </is>
+      </c>
+      <c r="M2" s="12" t="inlineStr">
+        <is>
+          <t>อายุสัญญาณ (แท่ง)</t>
+        </is>
+      </c>
+      <c r="N2" s="12" t="inlineStr">
+        <is>
+          <t>ห่าง EMA26 %</t>
+        </is>
+      </c>
+      <c r="O2" s="12" t="inlineStr">
+        <is>
+          <t>ผลตอบแทน 20 วัน %</t>
+        </is>
+      </c>
+      <c r="P2" s="12" t="inlineStr">
+        <is>
+          <t>ผลตอบแทน 60 วัน %</t>
+        </is>
+      </c>
+      <c r="Q2" s="12" t="inlineStr">
+        <is>
+          <t>จุดตัดขาดทุน (2ATR)</t>
+        </is>
+      </c>
+      <c r="R2" s="12" t="inlineStr">
+        <is>
+          <t>มูลค่าซื้อขายเฉลี่ย 25 วัน (ลบ.)</t>
+        </is>
+      </c>
+      <c r="S2" s="12" t="inlineStr">
+        <is>
+          <t>มูลค่าตลาด (พันลบ.)</t>
+        </is>
+      </c>
+      <c r="T2" s="12" t="inlineStr">
+        <is>
+          <t>กลุ่มธุรกิจ</t>
+        </is>
+      </c>
+      <c r="U2" s="12" t="inlineStr">
+        <is>
+          <t>คำเตือน</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>CPALL</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>zone3</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>zone4 -&gt; zone3</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="J3" s="8" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="L3" s="8" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="O3" s="8" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="P3" s="8" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="Q3" s="8" t="n">
+        <v>45.29</v>
+      </c>
+      <c r="R3" s="8" t="n">
+        <v>1532</v>
+      </c>
+      <c r="S3" s="8" t="n">
+        <v>417.7</v>
+      </c>
+      <c r="T3" s="7" t="inlineStr">
+        <is>
+          <t>Retail Trade</t>
+        </is>
+      </c>
+      <c r="U3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>zone3</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>zone4 -&gt; zone3</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="J4" s="8" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="L4" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="8" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="O4" s="8" t="n">
+        <v>-0.92</v>
+      </c>
+      <c r="P4" s="8" t="n">
+        <v>12.57</v>
+      </c>
+      <c r="Q4" s="8" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="R4" s="8" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="S4" s="8" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="T4" s="7" t="inlineStr">
+        <is>
+          <t>Consumer Services</t>
+        </is>
+      </c>
+      <c r="U4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>zone2</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>zone1 -&gt; zone2</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K5" s="10" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="L5" s="10" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="10" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="O5" s="10" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="P5" s="10" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="Q5" s="10" t="n">
+        <v>8.31</v>
+      </c>
+      <c r="R5" s="10" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="S5" s="10" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="T5" s="9" t="inlineStr">
+        <is>
+          <t>Health Services</t>
+        </is>
+      </c>
+      <c r="U5" s="9" t="inlineStr">
+        <is>
+          <t>beta สูง 1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>LH</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>zone3</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>zone2 -&gt; zone3</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="O6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="8" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="Q6" s="8" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="R6" s="8" t="n">
+        <v>133.9</v>
+      </c>
+      <c r="S6" s="8" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="T6" s="7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="U6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>TASCO</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>zone3</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>zone4 -&gt; zone3</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>-3</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="O7" s="8" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="P7" s="8" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="Q7" s="8" t="n">
+        <v>13.57</v>
+      </c>
+      <c r="R7" s="8" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="S7" s="8" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="T7" s="7" t="inlineStr">
+        <is>
+          <t>Non-Energy Minerals</t>
+        </is>
+      </c>
+      <c r="U7" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Z17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -11762,1400 +12300,1400 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr"/>
-      <c r="C2" s="12" t="n">
+      <c r="B2" s="13" t="inlineStr"/>
+      <c r="C2" s="14" t="n">
         <v>8.15</v>
       </c>
-      <c r="D2" s="12" t="n">
+      <c r="D2" s="14" t="n">
         <v>49.8</v>
       </c>
-      <c r="E2" s="11" t="n">
+      <c r="E2" s="13" t="n">
         <v>65</v>
       </c>
-      <c r="F2" s="12" t="n">
+      <c r="F2" s="14" t="n">
         <v>64.2</v>
       </c>
-      <c r="G2" s="12" t="n">
+      <c r="G2" s="14" t="n">
         <v>53.2</v>
       </c>
-      <c r="H2" s="12" t="n">
+      <c r="H2" s="14" t="n">
         <v>22.5</v>
       </c>
-      <c r="I2" s="12" t="n">
+      <c r="I2" s="14" t="n">
         <v>77.90000000000001</v>
       </c>
-      <c r="J2" s="12" t="n">
+      <c r="J2" s="14" t="n">
         <v>6.52</v>
       </c>
-      <c r="K2" s="12" t="n">
+      <c r="K2" s="14" t="n">
         <v>7.95</v>
       </c>
-      <c r="L2" s="12" t="n">
+      <c r="L2" s="14" t="n">
         <v>1.4</v>
       </c>
-      <c r="M2" s="12" t="n">
+      <c r="M2" s="14" t="n">
         <v>3.6</v>
       </c>
-      <c r="N2" s="12" t="n">
+      <c r="N2" s="14" t="n">
         <v>1.3</v>
       </c>
-      <c r="O2" s="11" t="inlineStr">
+      <c r="O2" s="13" t="inlineStr">
         <is>
           <t>zone3</t>
         </is>
       </c>
-      <c r="P2" s="11" t="inlineStr">
+      <c r="P2" s="13" t="inlineStr">
         <is>
           <t>zone2 -&gt; zone3</t>
         </is>
       </c>
-      <c r="Q2" s="12" t="n">
+      <c r="Q2" s="14" t="n">
         <v>7.78</v>
       </c>
-      <c r="R2" s="12" t="n">
+      <c r="R2" s="14" t="n">
         <v>7.78</v>
       </c>
-      <c r="S2" s="12" t="n">
+      <c r="S2" s="14" t="n">
         <v>4.58</v>
       </c>
-      <c r="T2" s="12" t="n">
+      <c r="T2" s="14" t="n">
         <v>2.29</v>
       </c>
-      <c r="U2" s="12" t="n">
+      <c r="U2" s="14" t="n">
         <v>102.6</v>
       </c>
-      <c r="V2" s="12" t="n">
+      <c r="V2" s="14" t="n">
         <v>25.3</v>
       </c>
-      <c r="W2" s="12" t="n">
+      <c r="W2" s="14" t="n">
         <v>5.9</v>
       </c>
-      <c r="X2" s="12" t="n">
+      <c r="X2" s="14" t="n">
         <v>6.46</v>
       </c>
-      <c r="Y2" s="11" t="inlineStr">
+      <c r="Y2" s="13" t="inlineStr">
         <is>
           <t>Consumer Durables</t>
         </is>
       </c>
-      <c r="Z2" s="11" t="inlineStr"/>
+      <c r="Z2" s="13" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>AMATA</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr"/>
-      <c r="C3" s="12" t="n">
+      <c r="B3" s="13" t="inlineStr"/>
+      <c r="C3" s="14" t="n">
         <v>27.5</v>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D3" s="14" t="n">
         <v>49.5</v>
       </c>
-      <c r="E3" s="11" t="n">
+      <c r="E3" s="13" t="n">
         <v>85</v>
       </c>
-      <c r="F3" s="12" t="n">
+      <c r="F3" s="14" t="n">
         <v>51.5</v>
       </c>
-      <c r="G3" s="12" t="n">
+      <c r="G3" s="14" t="n">
         <v>72.40000000000001</v>
       </c>
-      <c r="H3" s="12" t="n">
+      <c r="H3" s="14" t="n">
         <v>29.4</v>
       </c>
-      <c r="I3" s="12" t="n">
+      <c r="I3" s="14" t="n">
         <v>56.4</v>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
         <v>-2.2</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="K3" s="14" t="n">
         <v>2.8</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>1.02</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>12.8</v>
       </c>
-      <c r="N3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>-8.699999999999999</v>
       </c>
-      <c r="O3" s="11" t="inlineStr">
+      <c r="O3" s="13" t="inlineStr">
         <is>
           <t>zone3</t>
         </is>
       </c>
-      <c r="P3" s="11" t="inlineStr">
+      <c r="P3" s="13" t="inlineStr">
         <is>
           <t>zone4 -&gt; zone3</t>
         </is>
       </c>
-      <c r="Q3" s="12" t="n">
+      <c r="Q3" s="14" t="n">
         <v>27.33</v>
       </c>
-      <c r="R3" s="12" t="n">
+      <c r="R3" s="14" t="n">
         <v>25.4</v>
       </c>
-      <c r="S3" s="12" t="n">
+      <c r="S3" s="14" t="n">
         <v>7.65</v>
       </c>
-      <c r="T3" s="12" t="n">
+      <c r="T3" s="14" t="n">
         <v>3.82</v>
       </c>
-      <c r="U3" s="12" t="n">
+      <c r="U3" s="14" t="n">
         <v>311.1</v>
       </c>
-      <c r="V3" s="12" t="n">
+      <c r="V3" s="14" t="n">
         <v>31.1</v>
       </c>
-      <c r="W3" s="12" t="n">
+      <c r="W3" s="14" t="n">
         <v>8.6</v>
       </c>
-      <c r="X3" s="12" t="n">
+      <c r="X3" s="14" t="n">
         <v>4.07</v>
       </c>
-      <c r="Y3" s="11" t="inlineStr">
+      <c r="Y3" s="13" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="Z3" s="11" t="inlineStr">
+      <c r="Z3" s="13" t="inlineStr">
         <is>
           <t>งบออกใน 8 วัน | RSI divergence ขาลง | แรงรายใหญ่แผ่วลง</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>SYNEX</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr"/>
-      <c r="C4" s="12" t="n">
+      <c r="B4" s="13" t="inlineStr"/>
+      <c r="C4" s="14" t="n">
         <v>9.65</v>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="14" t="n">
         <v>40.5</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="13" t="n">
         <v>75</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="14" t="n">
         <v>56.4</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="14" t="n">
         <v>51.1</v>
       </c>
-      <c r="H4" s="12" t="n">
+      <c r="H4" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="I4" s="12" t="n">
+      <c r="I4" s="14" t="n">
         <v>84.7</v>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
         <v>6.92</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="K4" s="14" t="n">
         <v>10.29</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>0.42</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="M4" s="14" t="n">
         <v>1.9</v>
       </c>
-      <c r="N4" s="12" t="n">
+      <c r="N4" s="14" t="n">
         <v>-3.2</v>
       </c>
-      <c r="O4" s="11" t="inlineStr">
+      <c r="O4" s="13" t="inlineStr">
         <is>
           <t>zone3</t>
         </is>
       </c>
-      <c r="P4" s="11" t="inlineStr">
+      <c r="P4" s="13" t="inlineStr">
         <is>
           <t>zone2 -&gt; zone3</t>
         </is>
       </c>
-      <c r="Q4" s="12" t="n">
+      <c r="Q4" s="14" t="n">
         <v>9.44</v>
       </c>
-      <c r="R4" s="12" t="n">
+      <c r="R4" s="14" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="S4" s="12" t="n">
+      <c r="S4" s="14" t="n">
         <v>4.63</v>
       </c>
-      <c r="T4" s="12" t="n">
+      <c r="T4" s="14" t="n">
         <v>2.31</v>
       </c>
-      <c r="U4" s="12" t="n">
+      <c r="U4" s="14" t="n">
         <v>31.3</v>
       </c>
-      <c r="V4" s="12" t="n">
+      <c r="V4" s="14" t="n">
         <v>8.1</v>
       </c>
-      <c r="W4" s="12" t="n">
+      <c r="W4" s="14" t="n">
         <v>10.2</v>
       </c>
-      <c r="X4" s="12" t="n">
+      <c r="X4" s="14" t="n">
         <v>5.03</v>
       </c>
-      <c r="Y4" s="11" t="inlineStr">
+      <c r="Y4" s="13" t="inlineStr">
         <is>
           <t>Distribution Services</t>
         </is>
       </c>
-      <c r="Z4" s="11" t="inlineStr"/>
+      <c r="Z4" s="13" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>BH</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>B-Breakout</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="14" t="n">
         <v>186.5</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="14" t="n">
         <v>39.5</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="14" t="n">
         <v>54.4</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="14" t="n">
         <v>54.3</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="14" t="n">
         <v>15.8</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="14" t="n">
         <v>27.5</v>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="14" t="n">
         <v>-1.2</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="K5" s="14" t="n">
         <v>-0.8</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <v>1.9</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="M5" s="14" t="n">
         <v>4.7</v>
       </c>
-      <c r="N5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>1.4</v>
       </c>
-      <c r="O5" s="11" t="inlineStr">
+      <c r="O5" s="13" t="inlineStr">
         <is>
           <t>zone3</t>
         </is>
       </c>
-      <c r="P5" s="11" t="inlineStr">
+      <c r="P5" s="13" t="inlineStr">
         <is>
           <t>zone4 -&gt; zone3</t>
         </is>
       </c>
-      <c r="Q5" s="12" t="n">
+      <c r="Q5" s="14" t="n">
         <v>184.21</v>
       </c>
-      <c r="R5" s="12" t="n">
+      <c r="R5" s="14" t="n">
         <v>179.19</v>
       </c>
-      <c r="S5" s="12" t="n">
+      <c r="S5" s="14" t="n">
         <v>3.92</v>
       </c>
-      <c r="T5" s="12" t="n">
+      <c r="T5" s="14" t="n">
         <v>1.96</v>
       </c>
-      <c r="U5" s="12" t="n">
+      <c r="U5" s="14" t="n">
         <v>734.7</v>
       </c>
-      <c r="V5" s="12" t="n">
+      <c r="V5" s="14" t="n">
         <v>145.5</v>
       </c>
-      <c r="W5" s="12" t="n">
+      <c r="W5" s="14" t="n">
         <v>21.4</v>
       </c>
-      <c r="X5" s="12" t="n">
+      <c r="X5" s="14" t="n">
         <v>2.73</v>
       </c>
-      <c r="Y5" s="11" t="inlineStr">
+      <c r="Y5" s="13" t="inlineStr">
         <is>
           <t>Health Services</t>
         </is>
       </c>
-      <c r="Z5" s="11" t="inlineStr"/>
+      <c r="Z5" s="13" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>CPALL</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>B-Breakout C-Pullback</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="14" t="n">
         <v>47</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="14" t="n">
         <v>38.4</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="13" t="n">
         <v>70</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="14" t="n">
         <v>52.6</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="14" t="n">
         <v>51.9</v>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="14" t="n">
         <v>10.6</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="14" t="n">
         <v>39.1</v>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
         <v>-2.42</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="K6" s="14" t="n">
         <v>0.53</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>1.01</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="M6" s="14" t="n">
         <v>1.9</v>
       </c>
-      <c r="N6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>-0.7</v>
       </c>
-      <c r="O6" s="11" t="inlineStr">
+      <c r="O6" s="13" t="inlineStr">
         <is>
           <t>zone3</t>
         </is>
       </c>
-      <c r="P6" s="11" t="inlineStr">
+      <c r="P6" s="13" t="inlineStr">
         <is>
           <t>zone4 -&gt; zone3</t>
         </is>
       </c>
-      <c r="Q6" s="12" t="n">
+      <c r="Q6" s="14" t="n">
         <v>46.73</v>
       </c>
-      <c r="R6" s="12" t="n">
+      <c r="R6" s="14" t="n">
         <v>45.29</v>
       </c>
-      <c r="S6" s="12" t="n">
+      <c r="S6" s="14" t="n">
         <v>3.64</v>
       </c>
-      <c r="T6" s="12" t="n">
+      <c r="T6" s="14" t="n">
         <v>1.82</v>
       </c>
-      <c r="U6" s="12" t="n">
+      <c r="U6" s="14" t="n">
         <v>1532</v>
       </c>
-      <c r="V6" s="12" t="n">
+      <c r="V6" s="14" t="n">
         <v>417.7</v>
       </c>
-      <c r="W6" s="12" t="n">
+      <c r="W6" s="14" t="n">
         <v>14.3</v>
       </c>
-      <c r="X6" s="12" t="n">
+      <c r="X6" s="14" t="n">
         <v>3.55</v>
       </c>
-      <c r="Y6" s="11" t="inlineStr">
+      <c r="Y6" s="13" t="inlineStr">
         <is>
           <t>Retail Trade</t>
         </is>
       </c>
-      <c r="Z6" s="11" t="inlineStr"/>
+      <c r="Z6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>TASCO</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>C-Pullback</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="14" t="n">
         <v>34.2</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="14" t="n">
         <v>52.9</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="14" t="n">
         <v>52.4</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="14" t="n">
         <v>61</v>
       </c>
-      <c r="J7" s="12" t="n">
+      <c r="J7" s="14" t="n">
         <v>0.15</v>
       </c>
-      <c r="K7" s="12" t="n">
+      <c r="K7" s="14" t="n">
         <v>3.7</v>
       </c>
-      <c r="L7" s="12" t="n">
+      <c r="L7" s="14" t="n">
         <v>0.67</v>
       </c>
-      <c r="M7" s="12" t="n">
+      <c r="M7" s="14" t="n">
         <v>2.3</v>
       </c>
-      <c r="N7" s="12" t="n">
+      <c r="N7" s="14" t="n">
         <v>-3</v>
       </c>
-      <c r="O7" s="11" t="inlineStr">
+      <c r="O7" s="13" t="inlineStr">
         <is>
           <t>zone3</t>
         </is>
       </c>
-      <c r="P7" s="11" t="inlineStr">
+      <c r="P7" s="13" t="inlineStr">
         <is>
           <t>zone4 -&gt; zone3</t>
         </is>
       </c>
-      <c r="Q7" s="12" t="n">
+      <c r="Q7" s="14" t="n">
         <v>13.91</v>
       </c>
-      <c r="R7" s="12" t="n">
+      <c r="R7" s="14" t="n">
         <v>13.57</v>
       </c>
-      <c r="S7" s="12" t="n">
+      <c r="S7" s="14" t="n">
         <v>3.11</v>
       </c>
-      <c r="T7" s="12" t="n">
+      <c r="T7" s="14" t="n">
         <v>1.55</v>
       </c>
-      <c r="U7" s="12" t="n">
+      <c r="U7" s="14" t="n">
         <v>57.6</v>
       </c>
-      <c r="V7" s="12" t="n">
+      <c r="V7" s="14" t="n">
         <v>21.8</v>
       </c>
-      <c r="W7" s="12" t="n">
+      <c r="W7" s="14" t="n">
         <v>19.2</v>
       </c>
-      <c r="X7" s="12" t="n">
+      <c r="X7" s="14" t="n">
         <v>7.25</v>
       </c>
-      <c r="Y7" s="11" t="inlineStr">
+      <c r="Y7" s="13" t="inlineStr">
         <is>
           <t>Non-Energy Minerals</t>
         </is>
       </c>
-      <c r="Z7" s="11" t="inlineStr"/>
+      <c r="Z7" s="13" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>C-Pullback</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="14" t="n">
         <v>21.5</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="14" t="n">
         <v>31.6</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="14" t="n">
         <v>51.1</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="14" t="n">
         <v>52.8</v>
       </c>
-      <c r="H8" s="12" t="n">
+      <c r="H8" s="14" t="n">
         <v>25.4</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="14" t="n">
         <v>26.4</v>
       </c>
-      <c r="J8" s="12" t="n">
+      <c r="J8" s="14" t="n">
         <v>-0.92</v>
       </c>
-      <c r="K8" s="12" t="n">
+      <c r="K8" s="14" t="n">
         <v>-0.92</v>
       </c>
-      <c r="L8" s="12" t="n">
+      <c r="L8" s="14" t="n">
         <v>0.5</v>
       </c>
-      <c r="M8" s="12" t="n">
+      <c r="M8" s="14" t="n">
         <v>2.3</v>
       </c>
-      <c r="N8" s="12" t="n">
+      <c r="N8" s="14" t="n">
         <v>-1.5</v>
       </c>
-      <c r="O8" s="11" t="inlineStr">
+      <c r="O8" s="13" t="inlineStr">
         <is>
           <t>zone3</t>
         </is>
       </c>
-      <c r="P8" s="11" t="inlineStr">
+      <c r="P8" s="13" t="inlineStr">
         <is>
           <t>zone4 -&gt; zone3</t>
         </is>
       </c>
-      <c r="Q8" s="12" t="n">
+      <c r="Q8" s="14" t="n">
         <v>21.44</v>
       </c>
-      <c r="R8" s="12" t="n">
+      <c r="R8" s="14" t="n">
         <v>20.41</v>
       </c>
-      <c r="S8" s="12" t="n">
+      <c r="S8" s="14" t="n">
         <v>5.07</v>
       </c>
-      <c r="T8" s="12" t="n">
+      <c r="T8" s="14" t="n">
         <v>2.54</v>
       </c>
-      <c r="U8" s="12" t="n">
+      <c r="U8" s="14" t="n">
         <v>48.5</v>
       </c>
-      <c r="V8" s="12" t="n">
+      <c r="V8" s="14" t="n">
         <v>19.6</v>
       </c>
-      <c r="W8" s="12" t="n">
+      <c r="W8" s="14" t="n">
         <v>25.3</v>
       </c>
-      <c r="X8" s="12" t="n">
+      <c r="X8" s="14" t="n">
         <v>4.69</v>
       </c>
-      <c r="Y8" s="11" t="inlineStr">
+      <c r="Y8" s="13" t="inlineStr">
         <is>
           <t>Consumer Services</t>
         </is>
       </c>
-      <c r="Z8" s="11" t="inlineStr"/>
+      <c r="Z8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>LH</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>C-Pullback</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="14" t="n">
         <v>3.78</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="14" t="n">
         <v>28.7</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="14" t="n">
         <v>53.3</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="14" t="n">
         <v>50.2</v>
       </c>
-      <c r="H9" s="12" t="n">
+      <c r="H9" s="14" t="n">
         <v>16.1</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="14" t="n">
         <v>34.2</v>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="14" t="n">
         <v>-5</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="K9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="L9" s="14" t="n">
         <v>0.7</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="M9" s="14" t="n">
         <v>0.8</v>
       </c>
-      <c r="N9" s="12" t="n">
+      <c r="N9" s="14" t="n">
         <v>-0.7</v>
       </c>
-      <c r="O9" s="11" t="inlineStr">
+      <c r="O9" s="13" t="inlineStr">
         <is>
           <t>zone3</t>
         </is>
       </c>
-      <c r="P9" s="11" t="inlineStr">
+      <c r="P9" s="13" t="inlineStr">
         <is>
           <t>zone2 -&gt; zone3</t>
         </is>
       </c>
-      <c r="Q9" s="12" t="n">
+      <c r="Q9" s="14" t="n">
         <v>3.76</v>
       </c>
-      <c r="R9" s="12" t="n">
+      <c r="R9" s="14" t="n">
         <v>3.65</v>
       </c>
-      <c r="S9" s="12" t="n">
+      <c r="S9" s="14" t="n">
         <v>3.4</v>
       </c>
-      <c r="T9" s="12" t="n">
+      <c r="T9" s="14" t="n">
         <v>1.7</v>
       </c>
-      <c r="U9" s="12" t="n">
+      <c r="U9" s="14" t="n">
         <v>133.9</v>
       </c>
-      <c r="V9" s="12" t="n">
+      <c r="V9" s="14" t="n">
         <v>45.2</v>
       </c>
-      <c r="W9" s="12" t="n">
+      <c r="W9" s="14" t="n">
         <v>12.6</v>
       </c>
-      <c r="X9" s="12" t="n">
+      <c r="X9" s="14" t="n">
         <v>6.61</v>
       </c>
-      <c r="Y9" s="11" t="inlineStr">
+      <c r="Y9" s="13" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="Z9" s="11" t="inlineStr"/>
+      <c r="Z9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>STECON</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>C-Pullback</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="16" t="n">
         <v>17.7</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="16" t="n">
         <v>50.8</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="15" t="n">
         <v>65</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="16" t="n">
         <v>47.8</v>
       </c>
-      <c r="G10" s="14" t="n">
+      <c r="G10" s="16" t="n">
         <v>66.40000000000001</v>
       </c>
-      <c r="H10" s="14" t="n">
+      <c r="H10" s="16" t="n">
         <v>33.8</v>
       </c>
-      <c r="I10" s="14" t="n">
+      <c r="I10" s="16" t="n">
         <v>21.9</v>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="16" t="n">
         <v>0.01</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="K10" s="16" t="n">
         <v>-1.67</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="L10" s="16" t="n">
         <v>1.15</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="M10" s="16" t="n">
         <v>10.4</v>
       </c>
-      <c r="N10" s="14" t="n">
+      <c r="N10" s="16" t="n">
         <v>-10</v>
       </c>
-      <c r="O10" s="13" t="inlineStr">
+      <c r="O10" s="15" t="inlineStr">
         <is>
           <t>zone4</t>
         </is>
       </c>
-      <c r="P10" s="13" t="inlineStr">
+      <c r="P10" s="15" t="inlineStr">
         <is>
           <t>zone3 -&gt; zone4</t>
         </is>
       </c>
-      <c r="Q10" s="14" t="n">
+      <c r="Q10" s="16" t="n">
         <v>18.01</v>
       </c>
-      <c r="R10" s="14" t="n">
+      <c r="R10" s="16" t="n">
         <v>16.35</v>
       </c>
-      <c r="S10" s="14" t="n">
+      <c r="S10" s="16" t="n">
         <v>7.6</v>
       </c>
-      <c r="T10" s="14" t="n">
+      <c r="T10" s="16" t="n">
         <v>3.8</v>
       </c>
-      <c r="U10" s="14" t="n">
+      <c r="U10" s="16" t="n">
         <v>360</v>
       </c>
-      <c r="V10" s="14" t="n">
+      <c r="V10" s="16" t="n">
         <v>27.5</v>
       </c>
-      <c r="W10" s="14" t="n">
+      <c r="W10" s="16" t="n">
         <v>13.6</v>
       </c>
-      <c r="X10" s="14" t="n">
+      <c r="X10" s="16" t="n">
         <v>3.01</v>
       </c>
-      <c r="Y10" s="13" t="inlineStr">
+      <c r="Y10" s="15" t="inlineStr">
         <is>
           <t>Industrial Services</t>
         </is>
       </c>
-      <c r="Z10" s="13" t="inlineStr">
+      <c r="Z10" s="15" t="inlineStr">
         <is>
           <t>แรงรายใหญ่แผ่วลง | โซน RSI เพิ่งอ่อนลง</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>TRT</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr"/>
-      <c r="C11" s="14" t="n">
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="16" t="n">
         <v>13.6</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="16" t="n">
         <v>47.4</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="15" t="n">
         <v>75</v>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="F11" s="16" t="n">
         <v>48.5</v>
       </c>
-      <c r="G11" s="14" t="n">
+      <c r="G11" s="16" t="n">
         <v>75.90000000000001</v>
       </c>
-      <c r="H11" s="14" t="n">
+      <c r="H11" s="16" t="n">
         <v>58.8</v>
       </c>
-      <c r="I11" s="14" t="n">
+      <c r="I11" s="16" t="n">
         <v>74.7</v>
       </c>
-      <c r="J11" s="14" t="n">
+      <c r="J11" s="16" t="n">
         <v>5.18</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="K11" s="16" t="n">
         <v>7.09</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="L11" s="16" t="n">
         <v>1.12</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="M11" s="16" t="n">
         <v>20.7</v>
       </c>
-      <c r="N11" s="14" t="n">
+      <c r="N11" s="16" t="n">
         <v>-13.5</v>
       </c>
-      <c r="O11" s="13" t="inlineStr">
+      <c r="O11" s="15" t="inlineStr">
         <is>
           <t>zone4</t>
         </is>
       </c>
-      <c r="P11" s="13" t="inlineStr">
+      <c r="P11" s="15" t="inlineStr">
         <is>
           <t>zone3 -&gt; zone4</t>
         </is>
       </c>
-      <c r="Q11" s="14" t="n">
+      <c r="Q11" s="16" t="n">
         <v>13.84</v>
       </c>
-      <c r="R11" s="14" t="n">
+      <c r="R11" s="16" t="n">
         <v>12.08</v>
       </c>
-      <c r="S11" s="14" t="n">
+      <c r="S11" s="16" t="n">
         <v>11.15</v>
       </c>
-      <c r="T11" s="14" t="n">
+      <c r="T11" s="16" t="n">
         <v>5.58</v>
       </c>
-      <c r="U11" s="14" t="n">
+      <c r="U11" s="16" t="n">
         <v>57.7</v>
       </c>
-      <c r="V11" s="14" t="n">
+      <c r="V11" s="16" t="n">
         <v>4.4</v>
       </c>
-      <c r="W11" s="14" t="n">
+      <c r="W11" s="16" t="n">
         <v>18.1</v>
       </c>
-      <c r="X11" s="14" t="n">
+      <c r="X11" s="16" t="n">
         <v>2.43</v>
       </c>
-      <c r="Y11" s="13" t="inlineStr">
+      <c r="Y11" s="15" t="inlineStr">
         <is>
           <t>Producer Manufacturing</t>
         </is>
       </c>
-      <c r="Z11" s="13" t="inlineStr">
+      <c r="Z11" s="15" t="inlineStr">
         <is>
           <t>RSI divergence ขาลง | แรงรายใหญ่แผ่วลง | โซน RSI เพิ่งอ่อนลง</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>SAMART</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr"/>
-      <c r="C12" s="14" t="n">
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="16" t="n">
         <v>5.6</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="16" t="n">
         <v>40.8</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F12" s="16" t="n">
         <v>49.9</v>
       </c>
-      <c r="G12" s="14" t="n">
+      <c r="G12" s="16" t="n">
         <v>48.7</v>
       </c>
-      <c r="H12" s="14" t="n">
+      <c r="H12" s="16" t="n">
         <v>10.4</v>
       </c>
-      <c r="I12" s="14" t="n">
+      <c r="I12" s="16" t="n">
         <v>55.8</v>
       </c>
-      <c r="J12" s="14" t="n">
+      <c r="J12" s="16" t="n">
         <v>0.17</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="K12" s="16" t="n">
         <v>2.75</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="L12" s="16" t="n">
         <v>1.14</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="M12" s="16" t="n">
         <v>-0.4</v>
       </c>
-      <c r="N12" s="14" t="n">
+      <c r="N12" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="O12" s="13" t="inlineStr">
+      <c r="O12" s="15" t="inlineStr">
         <is>
           <t>zone1</t>
         </is>
       </c>
-      <c r="P12" s="13" t="inlineStr">
+      <c r="P12" s="15" t="inlineStr">
         <is>
           <t>zone2 -&gt; zone1</t>
         </is>
       </c>
-      <c r="Q12" s="14" t="n">
+      <c r="Q12" s="16" t="n">
         <v>5.6</v>
       </c>
-      <c r="R12" s="14" t="n">
+      <c r="R12" s="16" t="n">
         <v>5.27</v>
       </c>
-      <c r="S12" s="14" t="n">
+      <c r="S12" s="16" t="n">
         <v>5.97</v>
       </c>
-      <c r="T12" s="14" t="n">
+      <c r="T12" s="16" t="n">
         <v>2.99</v>
       </c>
-      <c r="U12" s="14" t="n">
+      <c r="U12" s="16" t="n">
         <v>11.1</v>
       </c>
-      <c r="V12" s="14" t="n">
+      <c r="V12" s="16" t="n">
         <v>5.8</v>
       </c>
-      <c r="W12" s="14" t="n">
+      <c r="W12" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="X12" s="14" t="n">
+      <c r="X12" s="16" t="n">
         <v>4.17</v>
       </c>
-      <c r="Y12" s="13" t="inlineStr">
+      <c r="Y12" s="15" t="inlineStr">
         <is>
           <t>Commercial Services</t>
         </is>
       </c>
-      <c r="Z12" s="13" t="inlineStr">
+      <c r="Z12" s="15" t="inlineStr">
         <is>
           <t>งบออกใน 7 วัน | โซน RSI เพิ่งอ่อนลง</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>BCPG</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr"/>
-      <c r="C13" s="14" t="n">
+      <c r="B13" s="15" t="inlineStr"/>
+      <c r="C13" s="16" t="n">
         <v>7.1</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="16" t="n">
         <v>27.7</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="15" t="n">
         <v>40</v>
       </c>
-      <c r="F13" s="14" t="n">
+      <c r="F13" s="16" t="n">
         <v>45.8</v>
       </c>
-      <c r="G13" s="14" t="n">
+      <c r="G13" s="16" t="n">
         <v>49.7</v>
       </c>
-      <c r="H13" s="14" t="n">
+      <c r="H13" s="16" t="n">
         <v>22.7</v>
       </c>
-      <c r="I13" s="14" t="n">
+      <c r="I13" s="16" t="n">
         <v>40.5</v>
       </c>
-      <c r="J13" s="14" t="n">
+      <c r="J13" s="16" t="n">
         <v>-3.25</v>
       </c>
-      <c r="K13" s="14" t="n">
+      <c r="K13" s="16" t="n">
         <v>0.71</v>
       </c>
-      <c r="L13" s="14" t="n">
+      <c r="L13" s="16" t="n">
         <v>1.22</v>
       </c>
-      <c r="M13" s="14" t="n">
+      <c r="M13" s="16" t="n">
         <v>-0</v>
       </c>
-      <c r="N13" s="14" t="n">
+      <c r="N13" s="16" t="n">
         <v>-5.3</v>
       </c>
-      <c r="O13" s="13" t="inlineStr">
+      <c r="O13" s="15" t="inlineStr">
         <is>
           <t>zone1</t>
         </is>
       </c>
-      <c r="P13" s="13" t="inlineStr">
+      <c r="P13" s="15" t="inlineStr">
         <is>
           <t>zone3 -&gt; zone1</t>
         </is>
       </c>
-      <c r="Q13" s="14" t="n">
+      <c r="Q13" s="16" t="n">
         <v>7.23</v>
       </c>
-      <c r="R13" s="14" t="n">
+      <c r="R13" s="16" t="n">
         <v>6.69</v>
       </c>
-      <c r="S13" s="14" t="n">
+      <c r="S13" s="16" t="n">
         <v>5.81</v>
       </c>
-      <c r="T13" s="14" t="n">
+      <c r="T13" s="16" t="n">
         <v>2.9</v>
       </c>
-      <c r="U13" s="14" t="n">
+      <c r="U13" s="16" t="n">
         <v>82.5</v>
       </c>
-      <c r="V13" s="14" t="n">
+      <c r="V13" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="W13" s="14" t="n">
+      <c r="W13" s="16" t="n">
         <v>14.9</v>
       </c>
-      <c r="X13" s="14" t="n">
+      <c r="X13" s="16" t="n">
         <v>4.76</v>
       </c>
-      <c r="Y13" s="13" t="inlineStr">
+      <c r="Y13" s="15" t="inlineStr">
         <is>
           <t>Utilities</t>
         </is>
       </c>
-      <c r="Z13" s="13" t="inlineStr">
+      <c r="Z13" s="15" t="inlineStr">
         <is>
           <t>โซน RSI เพิ่งอ่อนลง</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>KCE</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr"/>
-      <c r="C14" s="14" t="n">
+      <c r="B14" s="15" t="inlineStr"/>
+      <c r="C14" s="16" t="n">
         <v>37.75</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="16" t="n">
         <v>26.7</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="15" t="n">
         <v>45</v>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="F14" s="16" t="n">
         <v>41.6</v>
       </c>
-      <c r="G14" s="14" t="n">
+      <c r="G14" s="16" t="n">
         <v>63.4</v>
       </c>
-      <c r="H14" s="14" t="n">
+      <c r="H14" s="16" t="n">
         <v>18.5</v>
       </c>
-      <c r="I14" s="14" t="n">
+      <c r="I14" s="16" t="n">
         <v>5.3</v>
       </c>
-      <c r="J14" s="14" t="n">
+      <c r="J14" s="16" t="n">
         <v>-8.58</v>
       </c>
-      <c r="K14" s="14" t="n">
+      <c r="K14" s="16" t="n">
         <v>-9.58</v>
       </c>
-      <c r="L14" s="14" t="n">
+      <c r="L14" s="16" t="n">
         <v>1.76</v>
       </c>
-      <c r="M14" s="14" t="n">
+      <c r="M14" s="16" t="n">
         <v>5.7</v>
       </c>
-      <c r="N14" s="14" t="n">
+      <c r="N14" s="16" t="n">
         <v>-6.5</v>
       </c>
-      <c r="O14" s="13" t="inlineStr">
+      <c r="O14" s="15" t="inlineStr">
         <is>
           <t>zone4</t>
         </is>
       </c>
-      <c r="P14" s="13" t="inlineStr">
+      <c r="P14" s="15" t="inlineStr">
         <is>
           <t>zone3 -&gt; zone4</t>
         </is>
       </c>
-      <c r="Q14" s="14" t="n">
+      <c r="Q14" s="16" t="n">
         <v>40.67</v>
       </c>
-      <c r="R14" s="14" t="n">
+      <c r="R14" s="16" t="n">
         <v>33.63</v>
       </c>
-      <c r="S14" s="14" t="n">
+      <c r="S14" s="16" t="n">
         <v>10.91</v>
       </c>
-      <c r="T14" s="14" t="n">
+      <c r="T14" s="16" t="n">
         <v>5.46</v>
       </c>
-      <c r="U14" s="14" t="n">
+      <c r="U14" s="16" t="n">
         <v>890.8</v>
       </c>
-      <c r="V14" s="14" t="n">
+      <c r="V14" s="16" t="n">
         <v>49</v>
       </c>
-      <c r="W14" s="14" t="n">
+      <c r="W14" s="16" t="n">
         <v>53.3</v>
       </c>
-      <c r="X14" s="14" t="n">
+      <c r="X14" s="16" t="n">
         <v>2.89</v>
       </c>
-      <c r="Y14" s="13" t="inlineStr">
+      <c r="Y14" s="15" t="inlineStr">
         <is>
           <t>Electronic Technology</t>
         </is>
       </c>
-      <c r="Z14" s="13" t="inlineStr">
+      <c r="Z14" s="15" t="inlineStr">
         <is>
           <t>RSI divergence ขาลง | โซน RSI เพิ่งอ่อนลง</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>IVL</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr"/>
-      <c r="C15" s="14" t="n">
+      <c r="B15" s="15" t="inlineStr"/>
+      <c r="C15" s="16" t="n">
         <v>21.8</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="16" t="n">
         <v>25.1</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="15" t="n">
         <v>40</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F15" s="16" t="n">
         <v>37.3</v>
       </c>
-      <c r="G15" s="14" t="n">
+      <c r="G15" s="16" t="n">
         <v>47.2</v>
       </c>
-      <c r="H15" s="14" t="n">
+      <c r="H15" s="16" t="n">
         <v>25.9</v>
       </c>
-      <c r="I15" s="14" t="n">
+      <c r="I15" s="16" t="n">
         <v>26.5</v>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="16" t="n">
         <v>-3.69</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="K15" s="16" t="n">
         <v>-0.91</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="L15" s="16" t="n">
         <v>2.67</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="M15" s="16" t="n">
         <v>-3.7</v>
       </c>
-      <c r="N15" s="14" t="n">
+      <c r="N15" s="16" t="n">
         <v>-11.3</v>
       </c>
-      <c r="O15" s="13" t="inlineStr">
+      <c r="O15" s="15" t="inlineStr">
         <is>
           <t>zone1</t>
         </is>
       </c>
-      <c r="P15" s="13" t="inlineStr">
+      <c r="P15" s="15" t="inlineStr">
         <is>
           <t>zone3 -&gt; zone1</t>
         </is>
       </c>
-      <c r="Q15" s="14" t="n">
+      <c r="Q15" s="16" t="n">
         <v>23.73</v>
       </c>
-      <c r="R15" s="14" t="n">
+      <c r="R15" s="16" t="n">
         <v>20.12</v>
       </c>
-      <c r="S15" s="14" t="n">
+      <c r="S15" s="16" t="n">
         <v>7.69</v>
       </c>
-      <c r="T15" s="14" t="n">
+      <c r="T15" s="16" t="n">
         <v>3.85</v>
       </c>
-      <c r="U15" s="14" t="n">
+      <c r="U15" s="16" t="n">
         <v>741</v>
       </c>
-      <c r="V15" s="14" t="n">
+      <c r="V15" s="16" t="n">
         <v>135.3</v>
       </c>
-      <c r="W15" s="13" t="n"/>
-      <c r="X15" s="14" t="n">
+      <c r="W15" s="15" t="n"/>
+      <c r="X15" s="16" t="n">
         <v>2.9</v>
       </c>
-      <c r="Y15" s="13" t="inlineStr">
+      <c r="Y15" s="15" t="inlineStr">
         <is>
           <t>Process Industries</t>
         </is>
       </c>
-      <c r="Z15" s="13" t="inlineStr">
+      <c r="Z15" s="15" t="inlineStr">
         <is>
           <t>งบออกใน 8 วัน | beta สูง 1.7 | แรงรายใหญ่แผ่วลง | โซน RSI เพิ่งอ่อนลง</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>EA</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr"/>
-      <c r="C16" s="14" t="n">
+      <c r="B16" s="15" t="inlineStr"/>
+      <c r="C16" s="16" t="n">
         <v>2.9</v>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="D16" s="16" t="n">
         <v>18.3</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="F16" s="14" t="n">
+      <c r="F16" s="16" t="n">
         <v>41</v>
       </c>
-      <c r="G16" s="14" t="n">
+      <c r="G16" s="16" t="n">
         <v>48.7</v>
       </c>
-      <c r="H16" s="14" t="n">
+      <c r="H16" s="16" t="n">
         <v>14.5</v>
       </c>
-      <c r="I16" s="14" t="n">
+      <c r="I16" s="16" t="n">
         <v>34.2</v>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="16" t="n">
         <v>-3.96</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="K16" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="L16" s="16" t="n">
         <v>0.82</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="M16" s="16" t="n">
         <v>-1.1</v>
       </c>
-      <c r="N16" s="14" t="n">
+      <c r="N16" s="16" t="n">
         <v>-5.6</v>
       </c>
-      <c r="O16" s="13" t="inlineStr">
+      <c r="O16" s="15" t="inlineStr">
         <is>
           <t>zone1</t>
         </is>
       </c>
-      <c r="P16" s="13" t="inlineStr">
+      <c r="P16" s="15" t="inlineStr">
         <is>
           <t>zone4 -&gt; zone1</t>
         </is>
       </c>
-      <c r="Q16" s="14" t="n">
+      <c r="Q16" s="16" t="n">
         <v>3.02</v>
       </c>
-      <c r="R16" s="14" t="n">
+      <c r="R16" s="16" t="n">
         <v>2.7</v>
       </c>
-      <c r="S16" s="14" t="n">
+      <c r="S16" s="16" t="n">
         <v>6.77</v>
       </c>
-      <c r="T16" s="14" t="n">
+      <c r="T16" s="16" t="n">
         <v>3.39</v>
       </c>
-      <c r="U16" s="14" t="n">
+      <c r="U16" s="16" t="n">
         <v>219.2</v>
       </c>
-      <c r="V16" s="14" t="n">
+      <c r="V16" s="16" t="n">
         <v>21.7</v>
       </c>
-      <c r="W16" s="13" t="n"/>
-      <c r="X16" s="14" t="n">
+      <c r="W16" s="15" t="n"/>
+      <c r="X16" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="Y16" s="13" t="inlineStr">
+      <c r="Y16" s="15" t="inlineStr">
         <is>
           <t>Utilities</t>
         </is>
       </c>
-      <c r="Z16" s="13" t="inlineStr">
+      <c r="Z16" s="15" t="inlineStr">
         <is>
           <t>งบออกใน 7 วัน | โซน RSI เพิ่งอ่อนลง</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>DELTA</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr"/>
-      <c r="C17" s="14" t="n">
+      <c r="B17" s="15" t="inlineStr"/>
+      <c r="C17" s="16" t="n">
         <v>264</v>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="D17" s="16" t="n">
         <v>17.1</v>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="F17" s="14" t="n">
+      <c r="F17" s="16" t="n">
         <v>28.9</v>
       </c>
-      <c r="G17" s="14" t="n">
+      <c r="G17" s="16" t="n">
         <v>44.9</v>
       </c>
-      <c r="H17" s="14" t="n">
+      <c r="H17" s="16" t="n">
         <v>28.5</v>
       </c>
-      <c r="I17" s="14" t="n">
+      <c r="I17" s="16" t="n">
         <v>1.6</v>
       </c>
-      <c r="J17" s="14" t="n">
+      <c r="J17" s="16" t="n">
         <v>-17.77</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="K17" s="16" t="n">
         <v>-18.77</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="L17" s="16" t="n">
         <v>2.55</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="M17" s="16" t="n">
         <v>-6.8</v>
       </c>
-      <c r="N17" s="14" t="n">
+      <c r="N17" s="16" t="n">
         <v>-7.8</v>
       </c>
-      <c r="O17" s="13" t="inlineStr">
+      <c r="O17" s="15" t="inlineStr">
         <is>
           <t>zone1</t>
         </is>
       </c>
-      <c r="P17" s="13" t="inlineStr">
+      <c r="P17" s="15" t="inlineStr">
         <is>
           <t>zone4 -&gt; zone1</t>
         </is>
       </c>
-      <c r="Q17" s="14" t="n">
+      <c r="Q17" s="16" t="n">
         <v>316.65</v>
       </c>
-      <c r="R17" s="14" t="n">
+      <c r="R17" s="16" t="n">
         <v>239.89</v>
       </c>
-      <c r="S17" s="14" t="n">
+      <c r="S17" s="16" t="n">
         <v>9.130000000000001</v>
       </c>
-      <c r="T17" s="14" t="n">
+      <c r="T17" s="16" t="n">
         <v>4.57</v>
       </c>
-      <c r="U17" s="14" t="n">
+      <c r="U17" s="16" t="n">
         <v>4338</v>
       </c>
-      <c r="V17" s="14" t="n">
+      <c r="V17" s="16" t="n">
         <v>3555</v>
       </c>
-      <c r="W17" s="14" t="n">
+      <c r="W17" s="16" t="n">
         <v>110.3</v>
       </c>
-      <c r="X17" s="14" t="n">
+      <c r="X17" s="16" t="n">
         <v>0.21</v>
       </c>
-      <c r="Y17" s="13" t="inlineStr">
+      <c r="Y17" s="15" t="inlineStr">
         <is>
           <t>Electronic Technology</t>
         </is>
       </c>
-      <c r="Z17" s="13" t="inlineStr">
+      <c r="Z17" s="15" t="inlineStr">
         <is>
           <t>beta สูง 2.0 | โซน RSI เพิ่งอ่อนลง</t>
         </is>

</xml_diff>